<commit_message>
Added multi-theme dashboard styling with Dark, Light and Premium Glass UI
</commit_message>
<xml_diff>
--- a/Data/Defects Database Sample.xlsx
+++ b/Data/Defects Database Sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Predictive_Defect_Management_Dashboard\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB3EC35-D4B6-4F63-9FD3-BBCB8C54FF29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42AD082D-45E7-4AA7-8A94-20F25196D9C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RandomDB" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18444" uniqueCount="2312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18444" uniqueCount="2313">
   <si>
     <t>DefectCode</t>
   </si>
@@ -7010,6 +7010,9 @@
   </si>
   <si>
     <t>DataNest</t>
+  </si>
+  <si>
+    <t>DefectStatus</t>
   </si>
 </sst>
 </file>
@@ -7436,7 +7439,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>2312</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>

</xml_diff>